<commit_message>
Add Loom script and checklist; say what a second run actually does
README no longer says "the second run adds zero rows". It now says the
second run produces identical output, same counts and same rows,
because each run rewrites data/out from the same inputs; it does not
deduplicate against earlier runs. CLAUDE.md and QA.md never used the
phrase.

08-loom/script.md is a shot-by-shot script ending at 4:58, with a five
second segment at 4:45 on what was not done: nothing sent, no credits
spent, the 98 synthetic rows labelled. 08-loom/checklist.md lists what
to close, what to check and what to open, in order.

The workbook's Read me tab gains a Spend line ($0) so that claim is on
screen, and the committed snapshot is rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02-lead-list/inboxkit-leads.xlsx
+++ b/02-lead-list/inboxkit-leads.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -484,84 +484,96 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tier A</t>
+          <t>Spend</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Tier A is unreachable because headcount and techstack cannot be sourced free.</t>
+          <t>$0. Nothing was sent and no paid API was called; config/scale.md has the detail.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Tier A</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Verified-valid contacts that passed every ICP check, highest score first. (39 rows)</t>
+          <t>Tier A is unreachable because headcount and techstack cannot be sourced free.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Needs contact</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Accounts that passed every ICP check but have no verified contact yet. (2 rows)</t>
+          <t>Verified-valid contacts that passed every ICP check, highest score first. (39 rows)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Held</t>
+          <t>Needs contact</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Catch-all addresses, held back until a second check. (8 rows)</t>
+          <t>Accounts that passed every ICP check but have no verified contact yet. (2 rows)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Rejects</t>
+          <t>Held</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Duplicates, rows that failed an ICP check, and bad emails, each with a reason. (43 rows)</t>
+          <t>Catch-all addresses, held back until a second check. (8 rows)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Suppressed</t>
+          <t>Rejects</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Customers, competitors and opt-outs, with the rule that matched. (8 rows)</t>
+          <t>Duplicates, rows that failed an ICP check, and bad emails, each with a reason. (43 rows)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Suppressed</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Customers, competitors and opt-outs, with the rule that matched. (8 rows)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Run log</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>One row per pipeline run: counts, mode, credits, seconds. It holds every run since the repo was started, including development runs; the final run is the last row. (65 rows)</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>One row per pipeline run: counts, mode, credits, seconds. It holds every run since the repo was started, including development runs; the final run is the last row. (73 rows)</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O66"/>
+  <dimension ref="A1:O74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -11763,6 +11775,430 @@
       </c>
       <c r="O66" t="inlineStr"/>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-10-25T14:55:43+00:00</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>icp_jobchangers.yaml</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>15</v>
+      </c>
+      <c r="E67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" t="n">
+        <v>3</v>
+      </c>
+      <c r="H67" t="n">
+        <v>12</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="n">
+        <v>3</v>
+      </c>
+      <c r="K67" t="n">
+        <v>1</v>
+      </c>
+      <c r="L67" t="n">
+        <v>6</v>
+      </c>
+      <c r="M67" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-10-25T14:55:44+00:00</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>icp.yaml</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>100</v>
+      </c>
+      <c r="E68" t="n">
+        <v>8</v>
+      </c>
+      <c r="F68" t="n">
+        <v>8</v>
+      </c>
+      <c r="G68" t="n">
+        <v>21</v>
+      </c>
+      <c r="H68" t="n">
+        <v>73</v>
+      </c>
+      <c r="I68" t="n">
+        <v>2</v>
+      </c>
+      <c r="J68" t="n">
+        <v>14</v>
+      </c>
+      <c r="K68" t="n">
+        <v>8</v>
+      </c>
+      <c r="L68" t="n">
+        <v>39</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-10-25T17:07:01+00:00</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>icp.yaml</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>100</v>
+      </c>
+      <c r="E69" t="n">
+        <v>8</v>
+      </c>
+      <c r="F69" t="n">
+        <v>8</v>
+      </c>
+      <c r="G69" t="n">
+        <v>21</v>
+      </c>
+      <c r="H69" t="n">
+        <v>73</v>
+      </c>
+      <c r="I69" t="n">
+        <v>2</v>
+      </c>
+      <c r="J69" t="n">
+        <v>14</v>
+      </c>
+      <c r="K69" t="n">
+        <v>8</v>
+      </c>
+      <c r="L69" t="n">
+        <v>39</v>
+      </c>
+      <c r="M69" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-10-25T17:07:02+00:00</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>icp_try.yaml</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>100</v>
+      </c>
+      <c r="E70" t="n">
+        <v>8</v>
+      </c>
+      <c r="F70" t="n">
+        <v>8</v>
+      </c>
+      <c r="G70" t="n">
+        <v>61</v>
+      </c>
+      <c r="H70" t="n">
+        <v>24</v>
+      </c>
+      <c r="I70" t="n">
+        <v>2</v>
+      </c>
+      <c r="J70" t="n">
+        <v>5</v>
+      </c>
+      <c r="K70" t="n">
+        <v>2</v>
+      </c>
+      <c r="L70" t="n">
+        <v>14</v>
+      </c>
+      <c r="M70" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-10-25T17:07:02+00:00</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>icp_try.yaml</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>100</v>
+      </c>
+      <c r="E71" t="n">
+        <v>8</v>
+      </c>
+      <c r="F71" t="n">
+        <v>8</v>
+      </c>
+      <c r="G71" t="n">
+        <v>35</v>
+      </c>
+      <c r="H71" t="n">
+        <v>56</v>
+      </c>
+      <c r="I71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J71" t="n">
+        <v>10</v>
+      </c>
+      <c r="K71" t="n">
+        <v>6</v>
+      </c>
+      <c r="L71" t="n">
+        <v>31</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-10-25T17:07:03+00:00</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>icp.yaml</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>100</v>
+      </c>
+      <c r="E72" t="n">
+        <v>8</v>
+      </c>
+      <c r="F72" t="n">
+        <v>8</v>
+      </c>
+      <c r="G72" t="n">
+        <v>21</v>
+      </c>
+      <c r="H72" t="n">
+        <v>73</v>
+      </c>
+      <c r="I72" t="n">
+        <v>2</v>
+      </c>
+      <c r="J72" t="n">
+        <v>14</v>
+      </c>
+      <c r="K72" t="n">
+        <v>8</v>
+      </c>
+      <c r="L72" t="n">
+        <v>39</v>
+      </c>
+      <c r="M72" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>0.06</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-10-25T17:10:25+00:00</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>icp_jobchangers.yaml</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>15</v>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" t="n">
+        <v>3</v>
+      </c>
+      <c r="H73" t="n">
+        <v>12</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="n">
+        <v>3</v>
+      </c>
+      <c r="K73" t="n">
+        <v>1</v>
+      </c>
+      <c r="L73" t="n">
+        <v>6</v>
+      </c>
+      <c r="M73" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>0.08</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-10-25T17:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>icp.yaml</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>100</v>
+      </c>
+      <c r="E74" t="n">
+        <v>8</v>
+      </c>
+      <c r="F74" t="n">
+        <v>8</v>
+      </c>
+      <c r="G74" t="n">
+        <v>21</v>
+      </c>
+      <c r="H74" t="n">
+        <v>73</v>
+      </c>
+      <c r="I74" t="n">
+        <v>2</v>
+      </c>
+      <c r="J74" t="n">
+        <v>14</v>
+      </c>
+      <c r="K74" t="n">
+        <v>8</v>
+      </c>
+      <c r="L74" t="n">
+        <v>39</v>
+      </c>
+      <c r="M74" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>